<commit_message>
fix: add request hotel link
</commit_message>
<xml_diff>
--- a/link_hotel_data_expanded.xlsx
+++ b/link_hotel_data_expanded.xlsx
@@ -2952,12 +2952,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>HOTEL &amp; APARTMENT VY VAN</t>
+          <t>Ocean Pearl Villa</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/amp-apartment-vy-van.html?aid=356938&amp;label=metagha-link-MRVN-hotel-10383270_dev-desktop_los-1_bw-10_dow-Wednesday_defdate-0_room-0_gstadt-2_rateid-0_aud-7380914326_gacid-21411118307_mcid-10_ppa-0_clrid-0_ad-1_gstkid-0_checkin-20250924_ppt-_lp-2704_r-12456579030551460187&amp;sid=44d60f09dd88b24d5cca2032942ebcb9&amp;all_sr_blocks=1038327003_376329923_2_0_0&amp;checkin=2025-09-24&amp;checkout=2025-09-25&amp;dest_id=10383270&amp;dest_type=hotel&amp;dist=0&amp;group_adults=2&amp;group_children=0&amp;hapos=1&amp;highlighted_blocks=1038327003_376329923_2_0_0&amp;hpos=1&amp;matching_block_id=1038327003_376329923_2_0_0&amp;no_rooms=1&amp;req_adults=2&amp;req_children=0&amp;room1=A%2CA&amp;sb_price_type=total&amp;sr_order=popularity&amp;sr_pri_blocks=1038327003_376329923_2_0_0__25000000&amp;srepoch=1757866195&amp;srpvid=1a2171941f9509a9&amp;type=total&amp;ucfs=1&amp;</t>
+          <t>https://www.booking.com/hotel/vn/ocean-pearl-villa-vung-tau.vi.html?aid=304142&amp;dest_id=-3733750&amp;dest_type=city&amp;checkin=2026-09-20&amp;checkout=2026-09-21&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: update crawl automation scheduled
</commit_message>
<xml_diff>
--- a/link_hotel_data_expanded.xlsx
+++ b/link_hotel_data_expanded.xlsx
@@ -3296,7 +3296,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B61"/>
+  <dimension ref="A1:B60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -3798,238 +3798,226 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Mac Valley DaLat Hotel</t>
+          <t>TALA Dalat Hotel</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/mac-dalat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/taladalat-thanh-pho-da-lat123.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>TALA Dalat Hotel</t>
+          <t>Dream Boutique Hotel</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/taladalat-thanh-pho-da-lat123.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/dream-boutique.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Dream Boutique Hotel</t>
+          <t>Evermist Resort DaLat</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/dream-boutique.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/phuong-nguyen-villa.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Evermist Resort DaLat</t>
+          <t>Laimeront Dalat Hotel &amp; Apartment</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/phuong-nguyen-villa.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/de-l-aimeront.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Laimeront Dalat Hotel &amp; Apartment</t>
+          <t>PINE VIEW Hotel Dalat</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/de-l-aimeront.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/pine-view-dalat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>PINE VIEW Hotel Dalat</t>
+          <t>Nature Hotel - Pham Hong Thai</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/pine-view-dalat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/le-marais-dalat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Nature Hotel - Pham Hong Thai</t>
+          <t>Best Western Premier Imperial Dalat</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/le-marais-dalat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/best-western-premier-imperial-dalat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Best Western Premier Imperial Dalat</t>
+          <t>La Chérie Boutique Hotel</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/best-western-premier-imperial-dalat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/la-cherie-thanh-pho-da-lat1.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>La Chérie Boutique Hotel</t>
+          <t>NIA Hotel</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/la-cherie-thanh-pho-da-lat1.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/nia.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>NIA Hotel</t>
+          <t>Olive Hotel Da Lat</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/nia.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/olive.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Olive Hotel Da Lat</t>
+          <t>NATURE LAND 2 - Song Anh Hotel Dalat</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/olive.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/song-anh-thanh-pho-da-lat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>NATURE LAND 2 - Song Anh Hotel Dalat</t>
+          <t>The Manor Villas Da Lat</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/song-anh-thanh-pho-da-lat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/the-manor-villas-da-lat-thanh-pho-da-lat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>The Manor Villas Da Lat</t>
+          <t>Sweet Lavender Hotel - Ngay chợ đêm Đà Lạt</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/the-manor-villas-da-lat-thanh-pho-da-lat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/sweet-lavender-lam-dong.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Sweet Lavender Hotel - Ngay chợ đêm Đà Lạt</t>
+          <t>The Gate Boutique Hotel Đà Lạt</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/sweet-lavender-lam-dong.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/the-gate-boutique-da-lat-thanh-pho-da-lat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>The Gate Boutique Hotel Đà Lạt</t>
+          <t>Nature Hotel and Suite</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/the-gate-boutique-da-lat-thanh-pho-da-lat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/nature-and-suite.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Nature Hotel and Suite</t>
+          <t>TP Dalat Hotel</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/nature-and-suite.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/tp-pineview-dalat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>TP Dalat Hotel</t>
+          <t>Lumina Premium- HT Boutique 2 - Đống Đa</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/tp-pineview-dalat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/lumina-dalat-premium.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Lumina Premium- HT Boutique 2 - Đống Đa</t>
+          <t>Nature Hotel - Luong The Vinh</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/lumina-dalat-premium.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/cozy-boutique.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Nature Hotel - Luong The Vinh</t>
+          <t>Bazan Dalat Hotel</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/vn/cozy-boutique.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>Bazan Dalat Hotel</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
         <is>
           <t>https://www.booking.com/hotel/vn/bazan-dalat-thanh-pho-da-lat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>

</xml_diff>

<commit_message>
feat: fix aux local crawl sampling
</commit_message>
<xml_diff>
--- a/link_hotel_data_expanded.xlsx
+++ b/link_hotel_data_expanded.xlsx
@@ -3296,7 +3296,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B61"/>
+  <dimension ref="A1:B60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -3798,238 +3798,226 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Mac Valley DaLat Hotel</t>
+          <t>TALA Dalat Hotel</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/mac-dalat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/taladalat-thanh-pho-da-lat123.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>TALA Dalat Hotel</t>
+          <t>Dream Boutique Hotel</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/taladalat-thanh-pho-da-lat123.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/dream-boutique.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Dream Boutique Hotel</t>
+          <t>Evermist Resort DaLat</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/dream-boutique.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/phuong-nguyen-villa.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Evermist Resort DaLat</t>
+          <t>Laimeront Dalat Hotel &amp; Apartment</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/phuong-nguyen-villa.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/de-l-aimeront.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Laimeront Dalat Hotel &amp; Apartment</t>
+          <t>PINE VIEW Hotel Dalat</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/de-l-aimeront.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/pine-view-dalat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>PINE VIEW Hotel Dalat</t>
+          <t>Nature Hotel - Pham Hong Thai</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/pine-view-dalat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/le-marais-dalat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Nature Hotel - Pham Hong Thai</t>
+          <t>Best Western Premier Imperial Dalat</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/le-marais-dalat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/best-western-premier-imperial-dalat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Best Western Premier Imperial Dalat</t>
+          <t>La Chérie Boutique Hotel</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/best-western-premier-imperial-dalat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/la-cherie-thanh-pho-da-lat1.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>La Chérie Boutique Hotel</t>
+          <t>NIA Hotel</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/la-cherie-thanh-pho-da-lat1.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/nia.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>NIA Hotel</t>
+          <t>Olive Hotel Da Lat</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/nia.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/olive.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Olive Hotel Da Lat</t>
+          <t>NATURE LAND 2 - Song Anh Hotel Dalat</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/olive.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/song-anh-thanh-pho-da-lat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>NATURE LAND 2 - Song Anh Hotel Dalat</t>
+          <t>The Manor Villas Da Lat</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/song-anh-thanh-pho-da-lat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/the-manor-villas-da-lat-thanh-pho-da-lat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>The Manor Villas Da Lat</t>
+          <t>Sweet Lavender Hotel - Ngay chợ đêm Đà Lạt</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/the-manor-villas-da-lat-thanh-pho-da-lat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/sweet-lavender-lam-dong.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Sweet Lavender Hotel - Ngay chợ đêm Đà Lạt</t>
+          <t>The Gate Boutique Hotel Đà Lạt</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/sweet-lavender-lam-dong.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/the-gate-boutique-da-lat-thanh-pho-da-lat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>The Gate Boutique Hotel Đà Lạt</t>
+          <t>Nature Hotel and Suite</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/the-gate-boutique-da-lat-thanh-pho-da-lat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/nature-and-suite.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Nature Hotel and Suite</t>
+          <t>TP Dalat Hotel</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/nature-and-suite.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/tp-pineview-dalat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>TP Dalat Hotel</t>
+          <t>Lumina Premium- HT Boutique 2 - Đống Đa</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/tp-pineview-dalat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/lumina-dalat-premium.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Lumina Premium- HT Boutique 2 - Đống Đa</t>
+          <t>Nature Hotel - Luong The Vinh</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/lumina-dalat-premium.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/cozy-boutique.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Nature Hotel - Luong The Vinh</t>
+          <t>Bazan Dalat Hotel</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/vn/cozy-boutique.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>Bazan Dalat Hotel</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
         <is>
           <t>https://www.booking.com/hotel/vn/bazan-dalat-thanh-pho-da-lat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>

</xml_diff>

<commit_message>
feat: sync dead_link fix + quality monitor from scraper-reliability
Bring scraper-reliability's dead_link circuit-break fix (2-probe
confirmation, hotel_link_health streak, evidence JSON) and
daily_quality_monitor.py onto deployment, alongside its existing
VPS proxy/wait-tuning fixes. Verified no conflicts with deployment-only
infra (docker-compose.yml, Dockerfile, driver.py proxy config, config.py
AVAILABILITY_WAIT_* settings) and 54/54 backend tests pass.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/link_hotel_data_expanded.xlsx
+++ b/link_hotel_data_expanded.xlsx
@@ -2952,12 +2952,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>HOTEL &amp; APARTMENT VY VAN</t>
+          <t>Ocean Pearl Villa</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/amp-apartment-vy-van.html?aid=356938&amp;label=metagha-link-MRVN-hotel-10383270_dev-desktop_los-1_bw-10_dow-Wednesday_defdate-0_room-0_gstadt-2_rateid-0_aud-7380914326_gacid-21411118307_mcid-10_ppa-0_clrid-0_ad-1_gstkid-0_checkin-20250924_ppt-_lp-2704_r-12456579030551460187&amp;sid=44d60f09dd88b24d5cca2032942ebcb9&amp;all_sr_blocks=1038327003_376329923_2_0_0&amp;checkin=2025-09-24&amp;checkout=2025-09-25&amp;dest_id=10383270&amp;dest_type=hotel&amp;dist=0&amp;group_adults=2&amp;group_children=0&amp;hapos=1&amp;highlighted_blocks=1038327003_376329923_2_0_0&amp;hpos=1&amp;matching_block_id=1038327003_376329923_2_0_0&amp;no_rooms=1&amp;req_adults=2&amp;req_children=0&amp;room1=A%2CA&amp;sb_price_type=total&amp;sr_order=popularity&amp;sr_pri_blocks=1038327003_376329923_2_0_0__25000000&amp;srepoch=1757866195&amp;srpvid=1a2171941f9509a9&amp;type=total&amp;ucfs=1&amp;</t>
+          <t>https://www.booking.com/hotel/vn/ocean-pearl-villa-vung-tau.vi.html?aid=304142&amp;dest_id=-3733750&amp;dest_type=city&amp;checkin=2026-09-20&amp;checkout=2026-09-21&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
@@ -3296,7 +3296,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B61"/>
+  <dimension ref="A1:B60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -3798,238 +3798,226 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Mac Valley DaLat Hotel</t>
+          <t>TALA Dalat Hotel</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/mac-dalat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/taladalat-thanh-pho-da-lat123.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>TALA Dalat Hotel</t>
+          <t>Dream Boutique Hotel</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/taladalat-thanh-pho-da-lat123.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/dream-boutique.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Dream Boutique Hotel</t>
+          <t>Evermist Resort DaLat</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/dream-boutique.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/phuong-nguyen-villa.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Evermist Resort DaLat</t>
+          <t>Laimeront Dalat Hotel &amp; Apartment</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/phuong-nguyen-villa.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/de-l-aimeront.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Laimeront Dalat Hotel &amp; Apartment</t>
+          <t>PINE VIEW Hotel Dalat</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/de-l-aimeront.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/pine-view-dalat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>PINE VIEW Hotel Dalat</t>
+          <t>Nature Hotel - Pham Hong Thai</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/pine-view-dalat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/le-marais-dalat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Nature Hotel - Pham Hong Thai</t>
+          <t>Best Western Premier Imperial Dalat</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/le-marais-dalat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/best-western-premier-imperial-dalat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Best Western Premier Imperial Dalat</t>
+          <t>La Chérie Boutique Hotel</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/best-western-premier-imperial-dalat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/la-cherie-thanh-pho-da-lat1.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>La Chérie Boutique Hotel</t>
+          <t>NIA Hotel</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/la-cherie-thanh-pho-da-lat1.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/nia.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>NIA Hotel</t>
+          <t>Olive Hotel Da Lat</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/nia.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/olive.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Olive Hotel Da Lat</t>
+          <t>NATURE LAND 2 - Song Anh Hotel Dalat</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/olive.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/song-anh-thanh-pho-da-lat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>NATURE LAND 2 - Song Anh Hotel Dalat</t>
+          <t>The Manor Villas Da Lat</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/song-anh-thanh-pho-da-lat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/the-manor-villas-da-lat-thanh-pho-da-lat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>The Manor Villas Da Lat</t>
+          <t>Sweet Lavender Hotel - Ngay chợ đêm Đà Lạt</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/the-manor-villas-da-lat-thanh-pho-da-lat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/sweet-lavender-lam-dong.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Sweet Lavender Hotel - Ngay chợ đêm Đà Lạt</t>
+          <t>The Gate Boutique Hotel Đà Lạt</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/sweet-lavender-lam-dong.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/the-gate-boutique-da-lat-thanh-pho-da-lat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>The Gate Boutique Hotel Đà Lạt</t>
+          <t>Nature Hotel and Suite</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/the-gate-boutique-da-lat-thanh-pho-da-lat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/nature-and-suite.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Nature Hotel and Suite</t>
+          <t>TP Dalat Hotel</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/nature-and-suite.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/tp-pineview-dalat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>TP Dalat Hotel</t>
+          <t>Lumina Premium- HT Boutique 2 - Đống Đa</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/tp-pineview-dalat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/lumina-dalat-premium.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Lumina Premium- HT Boutique 2 - Đống Đa</t>
+          <t>Nature Hotel - Luong The Vinh</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/vn/lumina-dalat-premium.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
+          <t>https://www.booking.com/hotel/vn/cozy-boutique.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Nature Hotel - Luong The Vinh</t>
+          <t>Bazan Dalat Hotel</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/vn/cozy-boutique.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>Bazan Dalat Hotel</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
         <is>
           <t>https://www.booking.com/hotel/vn/bazan-dalat-thanh-pho-da-lat.vi.html?aid=304142&amp;dest_id=-3712045&amp;dest_type=city&amp;checkin=2026-09-15&amp;checkout=2026-09-16&amp;group_adults=2&amp;group_children=0&amp;no_rooms=1&amp;selected_currency=VND&amp;lang=vi</t>
         </is>

</xml_diff>